<commit_message>
fix+rerun: _is_bank_dcf forward-reference bug + 8 fresh ticker re-runs
Bug: _is_bank_dcf was computed at line ~3103 but referenced at lines 2229/2253
(quality EM premium + historical anchoring guards). Added early detection
block before first use — consistent with Rule 14 keywords/exclusions.

Re-ran against updated engine: CSCO HCA META MSFT NFLX TGT TSLA TSM
Score deltas: TSM +0.5, HCA +0.2, TSLA +0.2, TGT -0.2, CSCO -0.1

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/excel/CSCO_model.xlsx
+++ b/static/excel/CSCO_model.xlsx
@@ -7353,11 +7353,11 @@
         </is>
       </c>
       <c r="B5" s="43" t="n">
-        <v>466877.357564</v>
+        <v>474588.151745</v>
       </c>
       <c r="C5" s="44" t="inlineStr">
         <is>
-          <t>FMP marketCap  |  price $118.2</t>
+          <t>FMP marketCap  |  price $120.41</t>
         </is>
       </c>
     </row>
@@ -7443,7 +7443,7 @@
       </c>
       <c r="C12" s="44" t="inlineStr">
         <is>
-          <t>FRED series DGS10  |  latest: 2026-05-20</t>
+          <t>FRED series DGS10  |  latest: 2026-05-21</t>
         </is>
       </c>
     </row>
@@ -7526,7 +7526,7 @@
         </is>
       </c>
       <c r="B19" s="50" t="n">
-        <v>1.055</v>
+        <v>1.054</v>
       </c>
       <c r="C19" s="44">
         <f> unlevered × (1 + (1 − t) × D/E)</f>
@@ -7809,16 +7809,16 @@
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="54" t="inlineStr">
         <is>
-          <t>WACC  =  (E/V × Re)  +  (D/V × Rd × (1 − t))</t>
+          <t>WACC  =  MAX(8.5%, (E/V × Re) + (D/V × Rd × (1 − t)))</t>
         </is>
       </c>
       <c r="B44" s="55">
-        <f>B8*B28+B9*B37*(1-B41)</f>
+        <f>MAX(0.085, B8*B28+B9*B37*(1-B41))</f>
         <v/>
       </c>
       <c r="C44" s="56" t="inlineStr">
         <is>
-          <t>Used as discount rate in DCF tab</t>
+          <t>Floored 8.5% (D-001); raw formula below</t>
         </is>
       </c>
     </row>
@@ -8565,12 +8565,12 @@
       </c>
       <c r="G16" s="83" t="inlineStr">
         <is>
-          <t>61,755 — 63,334</t>
+          <t>61,899 — 63,132</t>
         </is>
       </c>
       <c r="H16" s="83" t="inlineStr">
         <is>
-          <t>64,458 — 71,695</t>
+          <t>64,110 — 71,309</t>
         </is>
       </c>
       <c r="I16" s="83" t="inlineStr">
@@ -8767,12 +8767,12 @@
       </c>
       <c r="G21" s="83" t="inlineStr">
         <is>
-          <t>18,634 — 19,110</t>
+          <t>18,677 — 19,049</t>
         </is>
       </c>
       <c r="H21" s="83" t="inlineStr">
         <is>
-          <t>19,449 — 21,633</t>
+          <t>19,344 — 21,516</t>
         </is>
       </c>
       <c r="I21" s="83" t="inlineStr">
@@ -9451,7 +9451,7 @@
         </is>
       </c>
       <c r="B38" s="103" t="n">
-        <v>10</v>
+        <v>11.4</v>
       </c>
       <c r="C38" s="101" t="n"/>
       <c r="D38" s="101" t="n"/>
@@ -9465,7 +9465,7 @@
       <c r="L38" s="101" t="n"/>
       <c r="M38" s="75" t="inlineStr">
         <is>
-          <t>Growth tier: LOW (3.4% 3yr avg rev growth).  Bear 8x / Base 10x / Bull 12x.  Override manually if needed.</t>
+          <t>Growth tier: LOW (3.4% 3yr avg rev growth).  Bear 9x / Base 11x / Bull 14x.  Override manually if needed.</t>
         </is>
       </c>
     </row>
@@ -9967,7 +9967,7 @@
         </is>
       </c>
       <c r="B61" s="114" t="n">
-        <v>118.2</v>
+        <v>120.41</v>
       </c>
       <c r="C61" s="106" t="n"/>
       <c r="D61" s="106" t="n"/>
@@ -10067,7 +10067,7 @@
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="116" t="inlineStr">
         <is>
-          <t>JS SCORECARD — CSCO  |  Master Prompt v2  |  22 May 2026  |  Sector bucket: Stable Compounder</t>
+          <t>JS SCORECARD — CSCO  |  Master Prompt v2  |  25 May 2026  |  Sector bucket: Stable Compounder</t>
         </is>
       </c>
     </row>
@@ -10584,7 +10584,7 @@
       </c>
       <c r="D22" s="132" t="inlineStr">
         <is>
-          <t>Current 26.8x  |  5yr avg 20.1x  |  DCF-implied 25.3x [ref only — not used as benchmark]  [+33% vs benchmark]  [trail=2.00 | no_fwd_data(fallback) | abs=4.0 → blended 40/40/20=2.40]  PEG≈839.50 (trailing_pe=26.8x / rev_cagr=3%, revenue proxy)</t>
+          <t>Current 26.8x  |  5yr avg 20.1x  |  DCF-implied 25.3x [ref only — not used as benchmark]  [+33% vs benchmark]  [trail=2.00 | fwd_pe=28.2x→1.16 | abs=4.0 → blended 40/40/20=2.07]  PEG=42.20 (fwd_pe=28.2x / eps_growth=67%)  [revision:Strong upgrade cycle→+0.50]</t>
         </is>
       </c>
       <c r="E22" s="139" t="inlineStr">
@@ -10593,7 +10593,7 @@
         </is>
       </c>
       <c r="F22" s="134" t="n">
-        <v>2.4</v>
+        <v>2.57</v>
       </c>
       <c r="G22" s="135">
         <f>IF(F22="",0,C22*F22*10)</f>
@@ -10601,7 +10601,7 @@
       </c>
       <c r="H22" s="136" t="inlineStr">
         <is>
-          <t>Current 26.8x  |  5yr avg 20.1x  |  DCF-implied 25.3x [ref only — not used as benchmark]  [+33% vs benchmark]  [trail=2.00 | no_fwd_data(fallback) | abs=4.0 → blended 40/40/20=2.40]  PEG≈839.50 (trailing_pe=26.8x / rev_cagr=3%, revenue proxy)</t>
+          <t>Current 26.8x  |  5yr avg 20.1x  |  DCF-implied 25.3x [ref only — not used as benchmark]  [+33% vs benchmark]  [trail=2.00 | fwd_pe=28.2x→1.16 | abs=4.0 → blended 40/40/20=2.07]  PEG=42.20 (fwd_pe=28.2x / eps_growth=67%)  [revision:Strong upgrade cycle→+0.50]</t>
         </is>
       </c>
     </row>
@@ -10621,7 +10621,7 @@
       </c>
       <c r="D23" s="132" t="inlineStr">
         <is>
-          <t>Current 20.6x  |  5yr avg 16.3x  |  DCF-implied 19.4x [ref only — not used as benchmark]  [+26% vs benchmark]  [trail=2.83 | no_fwd_data(fallback) | abs=7.5 → blended 40/40/20=3.77]</t>
+          <t>Current 20.6x  |  5yr avg 16.3x  |  DCF-implied 19.4x [ref only — not used as benchmark]  [+26% vs benchmark]  [trail=2.83 | fwd_pfcf=32.5x→0.00 | abs=7.5 → blended 40/40/20=2.63]</t>
         </is>
       </c>
       <c r="E23" s="139" t="inlineStr">
@@ -10630,7 +10630,7 @@
         </is>
       </c>
       <c r="F23" s="134" t="n">
-        <v>3.77</v>
+        <v>2.63</v>
       </c>
       <c r="G23" s="135">
         <f>IF(F23="",0,C23*F23*10)</f>
@@ -10638,7 +10638,7 @@
       </c>
       <c r="H23" s="136" t="inlineStr">
         <is>
-          <t>Current 20.6x  |  5yr avg 16.3x  |  DCF-implied 19.4x [ref only — not used as benchmark]  [+26% vs benchmark]  [trail=2.83 | no_fwd_data(fallback) | abs=7.5 → blended 40/40/20=3.77]</t>
+          <t>Current 20.6x  |  5yr avg 16.3x  |  DCF-implied 19.4x [ref only — not used as benchmark]  [+26% vs benchmark]  [trail=2.83 | fwd_pfcf=32.5x→0.00 | abs=7.5 → blended 40/40/20=2.63]</t>
         </is>
       </c>
     </row>

</xml_diff>